<commit_message>
Deployed 369c5f963 to fix-private-repos with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/fix-private-repos/catalog_summary.xlsx
+++ b/fix-private-repos/catalog_summary.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V5" t="n">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V16" t="n">
@@ -2163,9 +2163,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X16" t="n">
-        <v>2</v>
-      </c>
+      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -5426,7 +5424,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -5437,9 +5435,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X46" t="n">
-        <v>3</v>
-      </c>
+      <c r="X46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -7298,7 +7294,7 @@
       </c>
       <c r="U63" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V63" t="n">
@@ -9177,12 +9173,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9192,7 +9188,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9210,7 +9206,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9238,12 +9234,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9253,12 +9249,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9287,12 +9283,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9302,7 +9298,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9320,7 +9316,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9348,12 +9344,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9363,12 +9359,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -11358,7 +11354,7 @@
       </c>
       <c r="U100" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V100" t="n">
@@ -11369,9 +11365,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X100" t="n">
-        <v>3</v>
-      </c>
+      <c r="X100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11489,12 +11483,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11498,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11516,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11540,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11559,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11593,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11608,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11626,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11656,16 +11650,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11669,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11800,7 +11794,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11811,9 +11805,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X104" t="n">
-        <v>3</v>
-      </c>
+      <c r="X104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -12132,7 +12124,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -12143,9 +12135,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X107" t="n">
-        <v>3</v>
-      </c>
+      <c r="X107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -14918,7 +14908,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada.</t>
+          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14994,7 +14984,7 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V133" t="n">
@@ -15005,9 +14995,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="n">
-        <v>3</v>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -15766,7 +15754,7 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V140" t="n">
@@ -15777,9 +15765,7 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X140" t="n">
-        <v>3</v>
-      </c>
+      <c r="X140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -18190,7 +18176,7 @@
       </c>
       <c r="U162" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V162" t="n">
@@ -18201,9 +18187,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X162" t="n">
-        <v>3</v>
-      </c>
+      <c r="X162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -19436,7 +19420,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program, Provisional</t>
+          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program (Provisional)</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -19459,7 +19443,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -19512,7 +19496,7 @@
       </c>
       <c r="U174" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V174" t="n">
@@ -19523,7 +19507,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X174" t="inlineStr"/>
+      <c r="X174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -20119,7 +20105,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -20172,7 +20158,7 @@
       </c>
       <c r="U180" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V180" t="n">
@@ -20183,7 +20169,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X180" t="inlineStr"/>
+      <c r="X180" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -20559,7 +20547,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -20612,7 +20600,7 @@
       </c>
       <c r="U184" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V184" t="n">
@@ -20623,7 +20611,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="inlineStr"/>
+      <c r="X184" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -20733,9 +20723,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -20891,7 +20879,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -20944,7 +20932,7 @@
       </c>
       <c r="U187" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V187" t="n">
@@ -20955,9 +20943,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X187" t="n">
-        <v>3</v>
-      </c>
+      <c r="X187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -21716,7 +21702,7 @@
       </c>
       <c r="U194" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V194" t="n">
@@ -21727,9 +21713,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X194" t="n">
-        <v>3</v>
-      </c>
+      <c r="X194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -21828,7 +21812,7 @@
       </c>
       <c r="U195" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V195" t="n">
@@ -21839,9 +21823,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X195" t="n">
-        <v>2</v>
-      </c>
+      <c r="X195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -26996,7 +26978,7 @@
       </c>
       <c r="U242" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V242" t="inlineStr"/>
@@ -27100,7 +27082,7 @@
       </c>
       <c r="U243" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V243" t="n">
@@ -28686,7 +28668,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H258" t="b">
@@ -28752,7 +28734,7 @@
       </c>
       <c r="U258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V258" t="n">
@@ -28763,9 +28745,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X258" t="n">
-        <v>3</v>
-      </c>
+      <c r="X258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">

</xml_diff>